<commit_message>
chore: sync test31 project state and update submission docs
</commit_message>
<xml_diff>
--- a/modelData/pose_records.xlsx
+++ b/modelData/pose_records.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="12080"/>
+    <workbookView windowWidth="16060" windowHeight="5570"/>
   </bookViews>
   <sheets>
     <sheet name="pose_records" sheetId="1" r:id="rId1"/>
@@ -71,10 +71,10 @@
     <t>zone_01</t>
   </si>
   <si>
+    <t>zone_03</t>
+  </si>
+  <si>
     <t>zone_02</t>
-  </si>
-  <si>
-    <t>zone_03</t>
   </si>
   <si>
     <t>zone_04</t>
@@ -300,19 +300,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.79998168889431"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.5999938962981"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -324,19 +324,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.79998168889431"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.5999938962981"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -348,19 +348,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="6" tint="0.79998168889431"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.5999938962981"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -372,19 +372,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.79998168889431"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.5999938962981"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -396,19 +396,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.79998168889431"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.5999938962981"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -420,19 +420,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.79998168889431"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.5999938962981"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -474,7 +474,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4" tint="0.49998474074526"/>
       </bottom>
       <diagonal/>
     </border>
@@ -697,9 +697,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1236,9 +1234,16 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14" outlineLevelRow="5"/>
   <cols>
-    <col min="10" max="10" width="11.7272727272727"/>
-    <col min="11" max="11" width="12.8181818181818"/>
-    <col min="12" max="12" width="11.7272727272727"/>
+    <col min="1" max="1" width="17.4545454545455" customWidth="1"/>
+    <col min="2" max="2" width="8.45454545454546" customWidth="1"/>
+    <col min="3" max="3" width="14.4545454545455" customWidth="1"/>
+    <col min="4" max="4" width="8.45454545454546" customWidth="1"/>
+    <col min="5" max="5" width="7.45454545454545" customWidth="1"/>
+    <col min="6" max="8" width="8.45454545454546" customWidth="1"/>
+    <col min="9" max="9" width="7.45454545454545" customWidth="1"/>
+    <col min="10" max="10" width="11.4545454545455" customWidth="1"/>
+    <col min="11" max="11" width="12.4545454545455" customWidth="1"/>
+    <col min="12" max="12" width="11.4545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1357,7 +1362,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="1">
-        <v>46127.4494957986</v>
+        <v>46127.4508933333</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -1366,13 +1371,13 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <v>-0.1582</v>
+        <v>-1.5082</v>
       </c>
       <c r="E4">
-        <v>-1.476</v>
+        <v>-1.056</v>
       </c>
       <c r="F4">
-        <v>0.4259</v>
+        <v>-0.0241</v>
       </c>
       <c r="G4">
         <v>-0.5955</v>
@@ -1384,18 +1389,18 @@
         <v>1.3703</v>
       </c>
       <c r="J4">
-        <v>0.40819514</v>
+        <v>0.17385886</v>
       </c>
       <c r="K4">
-        <v>0.0762206</v>
+        <v>-0.54259241</v>
       </c>
       <c r="L4">
-        <v>0.83730734</v>
+        <v>0.79454355</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="1">
-        <v>46127.4508933333</v>
+        <v>46127.4494957986</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -1404,31 +1409,31 @@
         <v>1</v>
       </c>
       <c r="D5">
-        <v>-1.5082</v>
+        <v>0.0218</v>
       </c>
       <c r="E5">
-        <v>-1.056</v>
+        <v>-1.626</v>
       </c>
       <c r="F5">
-        <v>-0.0241</v>
+        <v>0.5159</v>
       </c>
       <c r="G5">
         <v>-0.5955</v>
       </c>
       <c r="H5">
-        <v>-1.6077</v>
+        <v>-1.6677</v>
       </c>
       <c r="I5">
-        <v>1.3703</v>
+        <v>1.4603</v>
       </c>
       <c r="J5">
-        <v>0.17385886</v>
+        <v>0.40819514</v>
       </c>
       <c r="K5">
-        <v>-0.54259241</v>
+        <v>0.0762206</v>
       </c>
       <c r="L5">
-        <v>0.79454355</v>
+        <v>0.83730734</v>
       </c>
     </row>
     <row r="6" spans="1:12">

</xml_diff>